<commit_message>
Build Xerox DCF and stock performance tabs
DCF: projection-assumption block (guidance-based 2026E, revenue decline,
synergy-driven margin, restructuring, depreciation, capex incl. lease
equipment, NWC) feeding the FCF build; WACC rebuilt (Kroll ERP, re-levered
comps beta, target 60/40 structure, 1L-implied cost of debt, 25% tax);
5.0x exit / 0% PGR terminal; debt and preferred in the bridge; every
assumption carries a sourced cell comment. Stock performance re-keyed to
XRX; external links removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xi44BzEwKbmnmxHD4YsneG
</commit_message>
<xml_diff>
--- a/Xerox_RX_Model_vClaude.xlsx
+++ b/Xerox_RX_Model_vClaude.xlsx
@@ -23,10 +23,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis &gt;" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="$XRX Comparable Companies" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="$FRSH DCF" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="$XRX DCF" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity Analysis" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Performance &gt; " sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="$FRSH Stock Performance" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="$XRX Stock Performance" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Football Field &gt;" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="$FRSH Valuation FF" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="24" state="visible" r:id="rId24"/>
@@ -92,9 +92,9 @@
     <definedName name="_xlnm.Print_Area" localSheetId="14">'Analysis &gt;'!$A$31</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="15">'Precedent Transactions'!$B$2:$Q$41,'Precedent Transactions'!$B$43:$Q$62</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="16">'$XRX Comparable Companies'!$B$2:$AG$44,'$XRX Comparable Companies'!$B$47:$M$66,'$XRX Comparable Companies'!$B$69:$K$92</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="17">'$FRSH DCF'!$B$2:$O$59,'$FRSH DCF'!$B$61:$O$113</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="17">'$XRX DCF'!$B$2:$O$59,'$XRX DCF'!$B$61:$O$112,'$XRX DCF'!$B$114:$O$131</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="19">'Stock Performance &gt; '!$B$1:$C$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="20">'$FRSH Stock Performance'!$B$2:$H$259,'$FRSH Stock Performance'!$J$9:$Q$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="20">'$XRX Stock Performance'!$B$2:$H$259,'$XRX Stock Performance'!$J$9:$Q$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="21">'Valuation Football Field &gt;'!$B$1:$C$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="22">'$FRSH Valuation FF'!$B$2:$I$48</definedName>
   </definedNames>
@@ -141,7 +141,7 @@
     <numFmt numFmtId="197" formatCode="[=1]&quot;Off&quot;;;&quot;On&quot;"/>
     <numFmt numFmtId="198" formatCode="mm/dd/yy;@"/>
   </numFmts>
-  <fonts count="82">
+  <fonts count="88">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -721,6 +721,40 @@
     <font>
       <name val="Garamond"/>
       <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <b val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <i val="1"/>
+      <color rgb="FF008000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Garamond"/>
+      <color rgb="FF008000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -1572,7 +1606,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="16"/>
     <xf numFmtId="44" fontId="17" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="1019">
+  <cellXfs count="1037">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -4098,6 +4132,28 @@
     <xf numFmtId="168" fontId="37" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="182" fontId="79" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="178" fontId="79" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="182" fontId="87" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="178" fontId="87" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="168" fontId="84" fillId="0" borderId="63" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="168" fontId="82" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="168" fontId="85" fillId="0" borderId="63" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="164" fontId="82" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="82" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="84" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="182" fontId="85" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="182" fontId="84" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="168" fontId="86" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="168" fontId="83" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="182" fontId="82" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="182" fontId="84" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="168" fontId="80" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="178" fontId="82" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="3"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6500,7 +6556,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'$FRSH Stock Performance'!$F$6</c:f>
+              <c:f>'$XRX Stock Performance'!$F$6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6526,7 +6582,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'$FRSH Stock Performance'!$C$7:$C$258</c:f>
+              <c:f>'$XRX Stock Performance'!$C$7:$C$258</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6537,7 +6593,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'$FRSH Stock Performance'!$F$7:$F$258</c:f>
+              <c:f>'$XRX Stock Performance'!$F$7:$F$258</c:f>
               <c:numCache>
                 <c:formatCode>##,##0.0%_);\(##,##0.0%\);"-"</c:formatCode>
                 <c:ptCount val="252"/>
@@ -7312,7 +7368,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'$FRSH Stock Performance'!$G$6</c:f>
+              <c:f>'$XRX Stock Performance'!$G$6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7335,7 +7391,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'$FRSH Stock Performance'!$C$7:$C$258</c:f>
+              <c:f>'$XRX Stock Performance'!$C$7:$C$258</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7346,7 +7402,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'$FRSH Stock Performance'!$G$7:$G$258</c:f>
+              <c:f>'$XRX Stock Performance'!$G$7:$G$258</c:f>
               <c:numCache>
                 <c:formatCode>##,##0.0%_);\(##,##0.0%\);"-"</c:formatCode>
                 <c:ptCount val="252"/>
@@ -9198,6 +9254,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Stephan Abedi</author>
+    <author>Claude</author>
   </authors>
   <commentList>
     <comment ref="J7" authorId="0" shapeId="0">
@@ -9210,29 +9267,54 @@
         <t>Includes deferred revenues.</t>
       </text>
     </comment>
+    <comment ref="N21" authorId="1" shapeId="0">
+      <text>
+        <t>Valuation date = 16-Oct-2026 (model date). 2026E UFCF is weighted by the remaining stub of the year.</t>
+      </text>
+    </comment>
     <comment ref="N22" authorId="0" shapeId="0">
       <text>
         <t>Fiscal year end for FRSH.</t>
       </text>
     </comment>
-    <comment ref="G26" authorId="0" shapeId="0">
+    <comment ref="G26" authorId="1" shapeId="0">
       <text>
-        <t>10-Y US Treasury Yield.</t>
+        <t>Risk-free rate: live FactSet 10-yr UST yield (TRYUS10Y). 10-yr was ~4.6-4.8% in Jul-Sep 2026 (Fed H.15 via YCharts). Kroll recommends the higher of 3.5% normalized or spot 20-yr.</t>
       </text>
     </comment>
-    <comment ref="G27" authorId="0" shapeId="0">
+    <comment ref="G27" authorId="1" shapeId="0">
       <text>
-        <t>Damodaran US Equity Risk Premium as of Jan 2026.</t>
+        <t>Equity risk premium 5.0% = Kroll recommended U.S. ERP (reaffirmed Jan-2026 and in the Sep-2026 Valuation Outlook), paired with the spot Treasury yield. Source: Kroll Cost of Capital (via BVWire, bvresources.com).</t>
       </text>
     </comment>
-    <comment ref="G28" authorId="0" shapeId="0">
+    <comment ref="G28" authorId="1" shapeId="0">
       <text>
-        <t>Beta was derived from a regression analysis using three measurement periods: 1-year daily, 3-year monthly, and 5-year weekly returns, with the median of the three used as the final input. See beta regression tab.</t>
+        <t>Re-levered beta: median UNLEVERED beta of the comp set ($XRX Comparable Companies col N, FactSet 5-yr) re-levered at the target D/E (60/40) and 25% tax. Falls back to 0.98 if FactSet is not loaded = Damodaran Office Equipment &amp; Services levered beta 1.33 at 32.5% D/(D+E), unlevered (Jan-2026, pages.stern.nyu.edu/~adamodar).</t>
       </text>
     </comment>
-    <comment ref="G37" authorId="0" shapeId="0">
+    <comment ref="G31" authorId="1" shapeId="0">
       <text>
-        <t>Using Damodaran Software sector effective tax rate as a simplifying assumption. Proper modeling would require a full NOL utilization schedule and a Section 382 analysis to determine the annual cap on NOL usage following the change of control. Given the complexity of this analysis, the DTA is held flat and cash taxes are modeled using the Damodaran.</t>
+        <t>Total debt = principal from the Capital Structure tab ($4,355mm at 2Q'26), not carrying value.</t>
+      </text>
+    </comment>
+    <comment ref="G33" authorId="1" shapeId="0">
+      <text>
+        <t>Target (normalized) capital structure of 60% debt / 40% equity rather than today's market weights (~92% debt at a ~$0.4bn equity cap), which reflect distress, not a sustainable structure. 60% ~ 3.0x net leverage on a ~5.0x EV/EBITDA business - where a reorganized Xerox could be levered (mgmt targets &lt;4x net by YE26). Above the 32% Office Equipment industry average (Damodaran, Jan-26) because ~$1.3bn of debt funds the captive finance book.</t>
+      </text>
+    </comment>
+    <comment ref="G35" authorId="1" shapeId="0">
+      <text>
+        <t>S&amp;P issuer CCC+ (restored from SD 16-Jun-26) / Moody's CFR Caa2 (Mar-26). See Capital Structure tab.</t>
+      </text>
+    </comment>
+    <comment ref="G36" authorId="1" shapeId="0">
+      <text>
+        <t>Spread ~8.5% over the 10-yr: Xerox's most senior traded paper, the 10.25% 1L notes due Oct-2030, quote ~88.6-91 (TRACE/Bondfish/BondBlox), i.e. ~12.8-13.5% YTM vs ~4.6-4.8% UST. Secured yield used because unsecured yields (2028s ~58c, 2029s ~41c) price default loss, not a going-concern cost of debt.</t>
+      </text>
+    </comment>
+    <comment ref="G37" authorId="1" shapeId="0">
+      <text>
+        <t>25% marginal tax rate: 21% U.S. federal + ~4% state/foreign blend. Xerox's reported adjusted rates are distorted by valuation allowances on losses (Q2'26 adj. ETR 31.3%; FY25 not meaningful), so a normalized marginal rate is used for NOPAT and the debt tax shield.</t>
       </text>
     </comment>
     <comment ref="G38" authorId="0" shapeId="0">
@@ -9240,14 +9322,89 @@
         <t>FRSH has no debt outstanding.</t>
       </text>
     </comment>
-    <comment ref="N45" authorId="0" shapeId="0">
+    <comment ref="N45" authorId="1" shapeId="0">
       <text>
-        <t>Nominal GDP growth in the US runs around 2-2.5% long-term. FRSH is a profitable, growing SaaS business with defensible recurring revenue so using the top end of that range is justified versus a slower growing or more commoditized business that might warrant 2% or below.</t>
+        <t>0.0% perpetuity growth: print volumes keep declining, partly offset by services and inflation pass-through; a no-growth terminal year is already generous for a secular-decline business. Sensitivity runs -1.0% to +1.0%.</t>
       </text>
     </comment>
-    <comment ref="G46" authorId="0" shapeId="0">
+    <comment ref="G46" authorId="1" shapeId="0">
       <text>
-        <t>Pulled from FactSet latest available.</t>
+        <t>5.0x EV/EBITDA exit: print/imaging peers trade ~3-6x (FactSet key comps: HP ~6x, Canon ~6x, Ricoh ~5x, Konica Minolta / Brother / Toshiba Tec ~4x, Seiko Epson ~3x). Xerox paid 4.7x LTM Adj. EBITDA for Lexmark (Dec-24). Damodaran Office Equipment &amp; Services avg 8.6x reflects healthier, un-levered U.S. names - too rich for a declining, distressed print franchise.</t>
+      </text>
+    </comment>
+    <comment ref="G52" authorId="1" shapeId="0">
+      <text>
+        <t>Deducts debt principal ($4,355mm) AND the $180mm Series A preferred liquidation preference (Capital Structure tab). Unfunded pension/OPEB (~$166mm/yr of contributions, excluded from UFCF) is a further debt-like claim not deducted here - deduct it for a fuller recovery waterfall.</t>
+      </text>
+    </comment>
+    <comment ref="G53" authorId="1" shapeId="0">
+      <text>
+        <t>Cash and cash equivalents at 30-Jun-26 ($495mm, Capital Structure tab).</t>
+      </text>
+    </comment>
+    <comment ref="G56" authorId="1" shapeId="0">
+      <text>
+        <t>Offline check of the base case (rf 4.7%, fallback beta): EV ~$3.45-3.7bn (~4.6x 2027E Adj. EBITDA) vs $4.36bn debt + $0.18bn preferred - i.e. equity is out of the money and the implied price is negative. In a restructuring context read the EV / debt coverage (~84% of principal) rather than the per-share value: secured debt ($2.05bn) is covered, unsecured is impaired - directionally consistent with unsecured bonds trading ~40-60c.</t>
+      </text>
+    </comment>
+    <comment ref="I71" authorId="1" shapeId="0">
+      <text>
+        <t>Axis centred on the 5.0x base exit multiple; step 0.5x. Re-centre if G46 changes (data-table headers cannot link to the input cell).</t>
+      </text>
+    </comment>
+    <comment ref="F74" authorId="1" shapeId="0">
+      <text>
+        <t>Axis centred on a ~12% WACC (rounded-up result of the inputs above with FactSet live); step 1.0%. Re-centre to G41 after FactSet refreshes.</t>
+      </text>
+    </comment>
+    <comment ref="J117" authorId="1" shapeId="0">
+      <text>
+        <t>2026E revenue = company guidance of ~$7.6bn (raised from &gt;$7.5bn on 30-Jul-26 with Q2 results). Includes a full year of Lexmark (acquired 1-Jul-25), hence +8% vs FY25 reported $7.0bn. Source: Xerox Q2'26 release / 8-K (sec.gov/Archives/edgar/data/1770450/000177045026000034).</t>
+      </text>
+    </comment>
+    <comment ref="K118" authorId="1" shapeId="0">
+      <text>
+        <t>2027E-2028E: -3.0%/yr. Q2'26 revenue was -6.5% pro forma (incl. Lexmark in both periods); office print page volumes are in structural decline and the only published 2028 street estimate ($7.44bn, ~-1%/yr) is a single-analyst outlier. -3% sits between the pro forma run-rate and that estimate, assuming IT/digital services partly offset print.</t>
+      </text>
+    </comment>
+    <comment ref="M118" authorId="1" shapeId="0">
+      <text>
+        <t>2029E-2030E: decline moderates to -2.5% as print mix shrinks and Lexmark A4 / services become a larger share. Still conservative vs flat; consistent with a secular-decline business with no new growth engine.</t>
+      </text>
+    </comment>
+    <comment ref="J119" authorId="1" shapeId="0">
+      <text>
+        <t>6.25% = midpoint of 2026 adjusted operating income guidance ($555-605mm) LESS the one-time $105mm IEEPA tariff-refund benefit = $475mm / $7.6bn. The refund is non-recurring, so it is excluded from the run-rate margin.</t>
+      </text>
+    </comment>
+    <comment ref="K119" authorId="1" shapeId="0">
+      <text>
+        <t>2027E 7.0% / 2028E+ 7.5%: Lexmark gross cost-synergy target raised to &gt;= $350mm (Q2'26), realized by end-2027. At $7.3bn revenue each $73mm of net synergy = ~1pt of margin; we credit only ~1.25pts of net expansion (synergies partly offset by price erosion, memory/oil cost inflation flagged by mgmt). Peers: Ricoh/Konica ~3-4%, Canon ~10% op. margin.</t>
+      </text>
+    </comment>
+    <comment ref="J121" authorId="1" shapeId="0">
+      <text>
+        <t>Restructuring &amp; related costs: LTM 2Q'26 $125mm (Income Statement Output). Treated as a real cash cost (excluded from 'adjusted' op. income by the company but still paid). Steps down as the Lexmark integration completes by end-2027, settling at ~$40mm/yr of ongoing footprint actions.</t>
+      </text>
+    </comment>
+    <comment ref="J123" authorId="1" shapeId="0">
+      <text>
+        <t>Depreciation ~3.8% of revenue: LTM D&amp;A of $415mm less $123mm amortization of intangibles (already excluded from adjusted op. income) = ~$292mm on $7.76bn LTM revenue. Held flat.</t>
+      </text>
+    </comment>
+    <comment ref="J125" authorId="1" shapeId="0">
+      <text>
+        <t>3.1% of revenue: LTM capex $99mm + investment in equipment on operating leases $141mm (rental fleet, reported inside operating cash flow) = $240mm on $7.76bn LTM revenue (Cash Flow Statement Output). Ties to 2026 guidance of ~$340mm OCF / ~$250mm FCF (~$90mm capex).</t>
+      </text>
+    </comment>
+    <comment ref="J127" authorId="1" shapeId="0">
+      <text>
+        <t>Operating NWC (excl. cash, debt, finance receivables) was -$206mm at 2Q'26 = -2.7% of LTM revenue (NWC tab). Held constant, so a shrinking revenue base releases slightly less negative NWC each year (small cash use). Finance receivables are treated as financing, not operating, and are excluded.</t>
+      </text>
+    </comment>
+    <comment ref="J128" authorId="1" shapeId="0">
+      <text>
+        <t>2026E change in NWC set to zero: the 1H26 seasonal build (-$239mm) is expected to reverse in 2H - mgmt's ~$340mm OCF guidance implies roughly flat full-year working capital.</t>
       </text>
     </comment>
   </commentList>
@@ -19339,7 +19496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P119"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="1.42578125" customWidth="1" min="1" max="1"/>
@@ -20083,7 +20240,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="15" customHeight="1">
       <c r="C30" s="532" t="inlineStr">
         <is>
@@ -20138,7 +20294,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1">
       <c r="C33" s="532" t="inlineStr">
         <is>
@@ -20193,7 +20348,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="15" customHeight="1">
       <c r="C36" s="532" t="inlineStr">
         <is>
@@ -20316,7 +20470,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43" ht="15" customHeight="1">
       <c r="J43" t="n"/>
       <c r="K43" t="n"/>
@@ -20656,61 +20809,13 @@
       <c r="J63" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1"/>
-    <row r="65"/>
     <row r="66" ht="15" customHeight="1"/>
     <row r="67" ht="15" customHeight="1"/>
-    <row r="68"/>
     <row r="69" ht="15" customHeight="1"/>
     <row r="70" ht="15" customHeight="1"/>
-    <row r="71"/>
     <row r="72" ht="15" customHeight="1"/>
     <row r="73" ht="15" customHeight="1"/>
     <row r="74" ht="15" customHeight="1"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="I24:I25 I60:I61" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -20733,7 +20838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF129"/>
+  <dimension ref="A1:AF93"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="1.42578125" customWidth="1" min="1" max="1"/>
@@ -20834,7 +20939,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="451" t="inlineStr">
         <is>
@@ -23634,7 +23738,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="15" customHeight="1">
       <c r="C38" s="532" t="inlineStr">
         <is>
@@ -24667,8 +24770,6 @@
       <c r="AC66" s="455" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1"/>
-    <row r="68"/>
-    <row r="69"/>
     <row r="70">
       <c r="B70" s="451" t="inlineStr">
         <is>
@@ -25746,42 +25847,6 @@
         </is>
       </c>
     </row>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="V21:V22" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
@@ -25804,7 +25869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O113"/>
+  <dimension ref="A1:O131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="1.42578125" customWidth="1" style="446" min="1" max="2"/>
@@ -25820,14 +25885,15 @@
         <v/>
       </c>
       <c r="B1" s="445">
-        <f>'[1]Cover Page'!A1</f>
+        <f>'Cover Page'!A1</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="C2" s="447">
-        <f>"$"&amp;'[1]Cover Page'!E16&amp;" Discounted Cash Flows"</f>
-        <v/>
+      <c r="C2" s="447" t="inlineStr">
+        <is>
+          <t>$XRX Discounted Cash Flows</t>
+        </is>
       </c>
       <c r="D2" s="447" t="n"/>
       <c r="E2" s="447" t="n"/>
@@ -25839,9 +25905,10 @@
       <c r="K2" s="465" t="n"/>
       <c r="L2" s="465" t="n"/>
       <c r="M2" s="465" t="n"/>
-      <c r="N2" s="448">
-        <f>'[1]Cover Page'!C2</f>
-        <v/>
+      <c r="N2" s="448" t="inlineStr">
+        <is>
+          <t>Xerox Holdings Corporation</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
@@ -25918,7 +25985,7 @@
       <c r="B7" s="685" t="n"/>
       <c r="C7" s="692" t="inlineStr">
         <is>
-          <t>EBIT</t>
+          <t>EBIT (Adj. Op. Income less Restructuring)</t>
         </is>
       </c>
       <c r="D7" s="693" t="n"/>
@@ -25927,20 +25994,25 @@
       <c r="G7" s="954" t="n"/>
       <c r="H7" s="955" t="n"/>
       <c r="I7" s="954" t="n"/>
-      <c r="J7" s="696" t="n">
-        <v>189</v>
-      </c>
-      <c r="K7" s="696" t="n">
-        <v>223</v>
-      </c>
-      <c r="L7" s="696" t="n">
-        <v>266</v>
-      </c>
-      <c r="M7" s="696" t="n">
-        <v>315</v>
-      </c>
-      <c r="N7" s="696" t="n">
-        <v>372</v>
+      <c r="J7" s="1019">
+        <f>J122</f>
+        <v/>
+      </c>
+      <c r="K7" s="1019">
+        <f>K122</f>
+        <v/>
+      </c>
+      <c r="L7" s="1019">
+        <f>L122</f>
+        <v/>
+      </c>
+      <c r="M7" s="1019">
+        <f>M122</f>
+        <v/>
+      </c>
+      <c r="N7" s="1019">
+        <f>N122</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
@@ -26018,7 +26090,7 @@
       <c r="B10" s="685" t="n"/>
       <c r="C10" s="958" t="inlineStr">
         <is>
-          <t>(+) Depreciation, Amortization, and Other Non-Cash Expenses</t>
+          <t>(+) Depreciation</t>
         </is>
       </c>
       <c r="D10" s="703" t="n"/>
@@ -26027,20 +26099,25 @@
       <c r="G10" s="703" t="n"/>
       <c r="H10" s="959" t="n"/>
       <c r="I10" s="959" t="n"/>
-      <c r="J10" s="960" t="n">
-        <v>15</v>
-      </c>
-      <c r="K10" s="960" t="n">
-        <v>18</v>
-      </c>
-      <c r="L10" s="960" t="n">
-        <v>20</v>
-      </c>
-      <c r="M10" s="960" t="n">
-        <v>23</v>
-      </c>
-      <c r="N10" s="960" t="n">
-        <v>27</v>
+      <c r="J10" s="1020">
+        <f>J124</f>
+        <v/>
+      </c>
+      <c r="K10" s="1020">
+        <f>K124</f>
+        <v/>
+      </c>
+      <c r="L10" s="1020">
+        <f>L124</f>
+        <v/>
+      </c>
+      <c r="M10" s="1020">
+        <f>M124</f>
+        <v/>
+      </c>
+      <c r="N10" s="1020">
+        <f>N124</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -26048,7 +26125,7 @@
       <c r="B11" s="685" t="n"/>
       <c r="C11" s="958" t="inlineStr">
         <is>
-          <t>(-) Capital Expenditures &amp; Purchases of Intangibles</t>
+          <t>(-) Capex incl. Equipment on Operating Leases</t>
         </is>
       </c>
       <c r="D11" s="703" t="n"/>
@@ -26057,20 +26134,25 @@
       <c r="G11" s="703" t="n"/>
       <c r="H11" s="703" t="n"/>
       <c r="I11" s="703" t="n"/>
-      <c r="J11" s="960" t="n">
-        <v>-22</v>
-      </c>
-      <c r="K11" s="960" t="n">
-        <v>-24</v>
-      </c>
-      <c r="L11" s="960" t="n">
-        <v>-27</v>
-      </c>
-      <c r="M11" s="960" t="n">
-        <v>-30</v>
-      </c>
-      <c r="N11" s="960" t="n">
-        <v>-34</v>
+      <c r="J11" s="1020">
+        <f>J126</f>
+        <v/>
+      </c>
+      <c r="K11" s="1020">
+        <f>K126</f>
+        <v/>
+      </c>
+      <c r="L11" s="1020">
+        <f>L126</f>
+        <v/>
+      </c>
+      <c r="M11" s="1020">
+        <f>M126</f>
+        <v/>
+      </c>
+      <c r="N11" s="1020">
+        <f>N126</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -26087,20 +26169,25 @@
       <c r="G12" s="703" t="n"/>
       <c r="H12" s="703" t="n"/>
       <c r="I12" s="703" t="n"/>
-      <c r="J12" s="960" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="960" t="n">
-        <v>15</v>
-      </c>
-      <c r="L12" s="960" t="n">
-        <v>33</v>
-      </c>
-      <c r="M12" s="960" t="n">
-        <v>49</v>
-      </c>
-      <c r="N12" s="960" t="n">
-        <v>65</v>
+      <c r="J12" s="1020">
+        <f>J128</f>
+        <v/>
+      </c>
+      <c r="K12" s="1020">
+        <f>K128</f>
+        <v/>
+      </c>
+      <c r="L12" s="1020">
+        <f>L128</f>
+        <v/>
+      </c>
+      <c r="M12" s="1020">
+        <f>M128</f>
+        <v/>
+      </c>
+      <c r="N12" s="1020">
+        <f>N128</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -26329,8 +26416,8 @@
       <c r="D20" s="500" t="n"/>
       <c r="E20" s="500" t="n"/>
       <c r="F20" s="500" t="n"/>
-      <c r="G20" s="722">
-        <f>'[1]$FRSH Comparable Companies'!F12</f>
+      <c r="G20" s="1021">
+        <f>'$XRX Comparable Companies'!F20</f>
         <v/>
       </c>
       <c r="H20" s="685" t="n"/>
@@ -26358,8 +26445,8 @@
       <c r="D21" s="500" t="n"/>
       <c r="E21" s="500" t="n"/>
       <c r="F21" s="500" t="n"/>
-      <c r="G21" s="971">
-        <f>'[1]$FRSH Comparable Companies'!G12</f>
+      <c r="G21" s="1022">
+        <f>'$XRX Comparable Companies'!G20</f>
         <v/>
       </c>
       <c r="H21" s="685" t="n"/>
@@ -26373,7 +26460,7 @@
       <c r="L21" s="500" t="n"/>
       <c r="M21" s="500" t="n"/>
       <c r="N21" s="972" t="n">
-        <v>46145</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -26428,14 +26515,14 @@
       <c r="B24" s="685" t="n"/>
       <c r="C24" s="730" t="inlineStr">
         <is>
-          <t>Weight of Equity</t>
+          <t>Weight of Equity (Target)</t>
         </is>
       </c>
       <c r="D24" s="731" t="n"/>
       <c r="E24" s="731" t="n"/>
       <c r="F24" s="731" t="n"/>
-      <c r="G24" s="974">
-        <f>G22/SUM($G$33,$G$22)</f>
+      <c r="G24" s="1023">
+        <f>1-G33</f>
         <v/>
       </c>
       <c r="H24" s="685" t="n"/>
@@ -26496,8 +26583,8 @@
       <c r="D27" s="500" t="n"/>
       <c r="E27" s="500" t="n"/>
       <c r="F27" s="500" t="n"/>
-      <c r="G27" s="965" t="n">
-        <v>0.0446</v>
+      <c r="G27" s="1024" t="n">
+        <v>0.05</v>
       </c>
       <c r="H27" s="685" t="n"/>
       <c r="I27" s="959" t="n"/>
@@ -26512,14 +26599,14 @@
       <c r="B28" s="685" t="n"/>
       <c r="C28" s="500" t="inlineStr">
         <is>
-          <t>Levered Beta</t>
+          <t>Levered Beta (re-levered at target D/E)</t>
         </is>
       </c>
       <c r="D28" s="500" t="n"/>
       <c r="E28" s="500" t="n"/>
       <c r="F28" s="500" t="n"/>
-      <c r="G28" s="971">
-        <f>'[1]$FRSH Beta Regression'!F9</f>
+      <c r="G28" s="1022">
+        <f>IFERROR('$XRX Comparable Companies'!N24,0.98)*(1+(1-G37)*(G33/G24))</f>
         <v/>
       </c>
       <c r="H28" s="677" t="n"/>
@@ -26580,8 +26667,9 @@
       <c r="D31" s="500" t="n"/>
       <c r="E31" s="500" t="n"/>
       <c r="F31" s="500" t="n"/>
-      <c r="G31" s="696" t="n">
-        <v>0</v>
+      <c r="G31" s="1021">
+        <f>'Capital Structure'!D24</f>
+        <v/>
       </c>
       <c r="H31" s="677" t="n"/>
       <c r="I31" s="685" t="n"/>
@@ -26612,15 +26700,14 @@
       <c r="B33" s="685" t="n"/>
       <c r="C33" s="730" t="inlineStr">
         <is>
-          <t>Weight of Debt</t>
+          <t>Weight of Debt (Target)</t>
         </is>
       </c>
       <c r="D33" s="731" t="n"/>
       <c r="E33" s="731" t="n"/>
       <c r="F33" s="731" t="n"/>
-      <c r="G33" s="974">
-        <f>IFERROR(G31/SUM($G$33,$G$24),0)</f>
-        <v/>
+      <c r="G33" s="1025" t="n">
+        <v>0.6</v>
       </c>
       <c r="H33" s="685" t="n"/>
       <c r="I33" s="959" t="n"/>
@@ -26657,9 +26744,9 @@
       <c r="D35" s="500" t="n"/>
       <c r="E35" s="500" t="n"/>
       <c r="F35" s="500" t="n"/>
-      <c r="G35" s="743" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="G35" s="1026" t="inlineStr">
+        <is>
+          <t>CCC+ / Caa2</t>
         </is>
       </c>
       <c r="H35" s="677" t="n"/>
@@ -26675,16 +26762,14 @@
       <c r="B36" s="685" t="n"/>
       <c r="C36" s="478" t="inlineStr">
         <is>
-          <t>Implied Credit Spread</t>
+          <t>Credit Spread over Risk-Free Rate</t>
         </is>
       </c>
       <c r="D36" s="500" t="n"/>
       <c r="E36" s="500" t="n"/>
       <c r="F36" s="500" t="n"/>
-      <c r="G36" s="744" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="G36" s="1027" t="n">
+        <v>0.08500000000000001</v>
       </c>
       <c r="H36" s="677" t="n"/>
       <c r="I36" s="685" t="n"/>
@@ -26705,9 +26790,8 @@
       <c r="D37" s="500" t="n"/>
       <c r="E37" s="500" t="n"/>
       <c r="F37" s="500" t="n"/>
-      <c r="G37" s="977">
-        <f>'[1]$FRSH Standalone 3SM'!M50</f>
-        <v/>
+      <c r="G37" s="1024" t="n">
+        <v>0.25</v>
       </c>
       <c r="H37" s="677" t="n"/>
       <c r="I37" s="685" t="n"/>
@@ -26728,8 +26812,9 @@
       <c r="D38" s="738" t="n"/>
       <c r="E38" s="738" t="n"/>
       <c r="F38" s="738" t="n"/>
-      <c r="G38" s="981" t="n">
-        <v>0</v>
+      <c r="G38" s="1028">
+        <f>(G26+G36)*(1-G37)</f>
+        <v/>
       </c>
       <c r="H38" s="685" t="n"/>
       <c r="I38" s="685" t="n"/>
@@ -26861,14 +26946,15 @@
       <c r="B45" s="685" t="n"/>
       <c r="C45" s="478" t="inlineStr">
         <is>
-          <t>Final Year Revenue</t>
+          <t>Final Year Adj. EBITDA (excl. IEEPA)</t>
         </is>
       </c>
       <c r="D45" s="500" t="n"/>
       <c r="E45" s="500" t="n"/>
       <c r="F45" s="500" t="n"/>
-      <c r="G45" s="696" t="n">
-        <v>1658</v>
+      <c r="G45" s="1019">
+        <f>N129</f>
+        <v/>
       </c>
       <c r="H45" s="685" t="n"/>
       <c r="I45" s="685" t="n"/>
@@ -26881,7 +26967,7 @@
       <c r="L45" s="500" t="n"/>
       <c r="M45" s="500" t="n"/>
       <c r="N45" s="982" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="O45" s="451" t="n"/>
     </row>
@@ -26890,14 +26976,14 @@
       <c r="B46" s="685" t="n"/>
       <c r="C46" s="500" t="inlineStr">
         <is>
-          <t>Exit Multiple</t>
+          <t>Exit EV / EBITDA Multiple</t>
         </is>
       </c>
       <c r="D46" s="500" t="n"/>
       <c r="E46" s="500" t="n"/>
       <c r="F46" s="983" t="n"/>
       <c r="G46" s="984" t="n">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="H46" s="677" t="n"/>
       <c r="I46" s="685" t="n"/>
@@ -27055,21 +27141,21 @@
       <c r="B52" s="685" t="n"/>
       <c r="C52" s="478" t="inlineStr">
         <is>
-          <t>(-) Debt</t>
+          <t>(-) Debt &amp; Preferred (principal)</t>
         </is>
       </c>
       <c r="D52" s="685" t="n"/>
       <c r="E52" s="685" t="n"/>
       <c r="F52" s="685" t="n"/>
       <c r="G52" s="956">
-        <f>-G31</f>
+        <f>-G31-'Capital Structure'!D27</f>
         <v/>
       </c>
       <c r="H52" s="685" t="n"/>
       <c r="I52" s="685" t="n"/>
       <c r="J52" s="478" t="inlineStr">
         <is>
-          <t>(-) Debt</t>
+          <t>(-) Debt &amp; Preferred (principal)</t>
         </is>
       </c>
       <c r="K52" s="685" t="n"/>
@@ -27091,8 +27177,8 @@
       <c r="D53" s="685" t="n"/>
       <c r="E53" s="685" t="n"/>
       <c r="F53" s="685" t="n"/>
-      <c r="G53" s="971">
-        <f>'[1]$FRSH Standalone 3SM'!I57</f>
+      <c r="G53" s="1022">
+        <f>-'Capital Structure'!D25</f>
         <v/>
       </c>
       <c r="H53" s="677" t="n"/>
@@ -27225,28 +27311,28 @@
       </c>
       <c r="C58" s="759" t="inlineStr">
         <is>
-          <t>Implied EV/NTM Adj. EBITDA Multiple</t>
+          <t>Implied EV / NTM (2027E) Adj. EBITDA</t>
         </is>
       </c>
       <c r="D58" s="760" t="n"/>
       <c r="E58" s="760" t="n"/>
       <c r="F58" s="760" t="n"/>
       <c r="G58" s="987">
-        <f>G51/'[1]$FRSH Standalone 3SM'!M38</f>
+        <f>G51/K129</f>
         <v/>
       </c>
       <c r="H58" s="685" t="n"/>
       <c r="I58" s="959" t="n"/>
       <c r="J58" s="759" t="inlineStr">
         <is>
-          <t>Implied EV/NTM Adj. EBITDA Multiple</t>
+          <t>Implied EV / NTM (2027E) Adj. EBITDA</t>
         </is>
       </c>
       <c r="K58" s="760" t="n"/>
       <c r="L58" s="760" t="n"/>
       <c r="M58" s="760" t="n"/>
       <c r="N58" s="987">
-        <f>N51/'[1]$FRSH Standalone 3SM'!M38</f>
+        <f>N51/K129</f>
         <v/>
       </c>
     </row>
@@ -27321,7 +27407,7 @@
         </is>
       </c>
       <c r="I65" s="988" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="K65" s="500" t="n"/>
       <c r="L65" s="764" t="n"/>
@@ -27341,7 +27427,7 @@
         </is>
       </c>
       <c r="I66" s="989" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="K66" s="500" t="n"/>
       <c r="L66" s="764" t="n"/>
@@ -27439,7 +27525,7 @@
         <v/>
       </c>
       <c r="I71" s="991" t="n">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="J71" s="990">
         <f>I71+$I$66</f>
@@ -27523,7 +27609,7 @@
         </is>
       </c>
       <c r="F74" s="988" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="G74" s="782" t="n">
         <v>13.26626339063693</v>
@@ -27669,7 +27755,7 @@
         <v/>
       </c>
       <c r="I81" s="991" t="n">
-        <v>1.9</v>
+        <v>5</v>
       </c>
       <c r="J81" s="990">
         <f>I81+$I$66</f>
@@ -27747,7 +27833,7 @@
         </is>
       </c>
       <c r="F84" s="988" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="G84" s="998" t="n">
         <v>0.5161443875013629</v>
@@ -27904,7 +27990,7 @@
         </is>
       </c>
       <c r="I92" s="1012" t="n">
-        <v>0.0025</v>
+        <v>0.005</v>
       </c>
       <c r="K92" s="500" t="n"/>
       <c r="L92" s="764" t="n"/>
@@ -27928,7 +28014,7 @@
     <row r="94" ht="15" customHeight="1">
       <c r="C94" s="769" t="inlineStr">
         <is>
-          <t>WACC and Exit Multiple Impact on PPS</t>
+          <t>WACC and Perpetuity Growth Rate Impact on PPS</t>
         </is>
       </c>
       <c r="D94" s="770" t="n"/>
@@ -27992,7 +28078,7 @@
         <v/>
       </c>
       <c r="I97" s="988" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="J97" s="993">
         <f>I97+$I$92</f>
@@ -28070,7 +28156,7 @@
         </is>
       </c>
       <c r="F100" s="988" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="G100" s="782" t="n">
         <v>22.92876405672628</v>
@@ -28148,7 +28234,7 @@
     <row r="104" ht="15" customHeight="1">
       <c r="C104" s="769" t="inlineStr">
         <is>
-          <t>WACC and Exit Multiple Impact on Implied Upside / (Downside)</t>
+          <t>WACC and Perpetuity Growth Rate Impact on Implied Upside / (Downside)</t>
         </is>
       </c>
       <c r="D104" s="770" t="n"/>
@@ -28212,7 +28298,7 @@
         <v/>
       </c>
       <c r="I107" s="988" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="J107" s="993">
         <f>I107+$I$92</f>
@@ -28290,7 +28376,7 @@
         </is>
       </c>
       <c r="F110" s="988" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="G110" s="998" t="n">
         <v>1.620430177911575</v>
@@ -28339,11 +28425,7 @@
       <c r="N111" s="764" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1">
-      <c r="A112" s="451" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="A112" s="451" t="n"/>
       <c r="B112" s="451" t="inlineStr">
         <is>
           <t>x</t>
@@ -28376,7 +28458,548 @@
       <c r="N112" s="764" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="451" t="inlineStr">
+      <c r="A113" s="451" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="677" t="n"/>
+      <c r="B115" s="677" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C115" s="678" t="inlineStr">
+        <is>
+          <t>Projection Assumptions (Base Case) - feeds the FCF build above</t>
+        </is>
+      </c>
+      <c r="D115" s="679" t="n"/>
+      <c r="E115" s="679" t="n"/>
+      <c r="F115" s="680" t="n"/>
+      <c r="G115" s="681" t="n"/>
+      <c r="H115" s="681" t="n"/>
+      <c r="I115" s="682" t="n"/>
+      <c r="J115" s="683" t="inlineStr">
+        <is>
+          <t>Projections</t>
+        </is>
+      </c>
+      <c r="K115" s="684" t="n"/>
+      <c r="L115" s="684" t="n"/>
+      <c r="M115" s="684" t="n"/>
+      <c r="N115" s="684" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="685" t="n"/>
+      <c r="B116" s="685" t="n"/>
+      <c r="C116" s="686" t="n"/>
+      <c r="D116" s="686" t="n"/>
+      <c r="E116" s="686" t="n"/>
+      <c r="F116" s="949" t="n"/>
+      <c r="G116" s="949" t="n"/>
+      <c r="H116" s="950" t="n"/>
+      <c r="I116" s="951" t="n"/>
+      <c r="J116" s="952">
+        <f>J6</f>
+        <v/>
+      </c>
+      <c r="K116" s="953">
+        <f>K6</f>
+        <v/>
+      </c>
+      <c r="L116" s="953">
+        <f>L6</f>
+        <v/>
+      </c>
+      <c r="M116" s="953">
+        <f>M6</f>
+        <v/>
+      </c>
+      <c r="N116" s="953">
+        <f>N6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="685" t="n"/>
+      <c r="B117" s="685" t="n"/>
+      <c r="C117" s="692" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D117" s="693" t="n"/>
+      <c r="E117" s="693" t="n"/>
+      <c r="F117" s="693" t="n"/>
+      <c r="G117" s="954" t="n"/>
+      <c r="H117" s="955" t="n"/>
+      <c r="I117" s="954" t="n"/>
+      <c r="J117" s="1029" t="n">
+        <v>7600</v>
+      </c>
+      <c r="K117" s="1030">
+        <f>J117*(1+K118)</f>
+        <v/>
+      </c>
+      <c r="L117" s="1030">
+        <f>K117*(1+L118)</f>
+        <v/>
+      </c>
+      <c r="M117" s="1030">
+        <f>L117*(1+M118)</f>
+        <v/>
+      </c>
+      <c r="N117" s="1030">
+        <f>M117*(1+N118)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="685" t="n"/>
+      <c r="B118" s="685" t="n"/>
+      <c r="C118" s="886" t="inlineStr">
+        <is>
+          <t>% Growth</t>
+        </is>
+      </c>
+      <c r="D118" s="685" t="n"/>
+      <c r="E118" s="685" t="n"/>
+      <c r="F118" s="685" t="n"/>
+      <c r="G118" s="685" t="n"/>
+      <c r="H118" s="685" t="n"/>
+      <c r="I118" s="685" t="n"/>
+      <c r="J118" s="1031">
+        <f>J117/'Income Statement Output'!H13-1</f>
+        <v/>
+      </c>
+      <c r="K118" s="1032" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="L118" s="1032" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="M118" s="1032" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="N118" s="1032" t="n">
+        <v>-0.025</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="685" t="n"/>
+      <c r="B119" s="685" t="n"/>
+      <c r="C119" s="886" t="inlineStr">
+        <is>
+          <t>Adj. Operating Margin (excl. IEEPA)</t>
+        </is>
+      </c>
+      <c r="D119" s="685" t="n"/>
+      <c r="E119" s="685" t="n"/>
+      <c r="F119" s="685" t="n"/>
+      <c r="G119" s="685" t="n"/>
+      <c r="H119" s="685" t="n"/>
+      <c r="I119" s="685" t="n"/>
+      <c r="J119" s="1032" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="K119" s="1032" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="L119" s="1032" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="M119" s="1032" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="N119" s="1032" t="n">
+        <v>0.075</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="685" t="n"/>
+      <c r="B120" s="685" t="n"/>
+      <c r="C120" s="692" t="inlineStr">
+        <is>
+          <t>Adj. Operating Income</t>
+        </is>
+      </c>
+      <c r="D120" s="693" t="n"/>
+      <c r="E120" s="693" t="n"/>
+      <c r="F120" s="693" t="n"/>
+      <c r="G120" s="954" t="n"/>
+      <c r="H120" s="955" t="n"/>
+      <c r="I120" s="954" t="n"/>
+      <c r="J120" s="1020">
+        <f>J117*J119</f>
+        <v/>
+      </c>
+      <c r="K120" s="1020">
+        <f>K117*K119</f>
+        <v/>
+      </c>
+      <c r="L120" s="1020">
+        <f>L117*L119</f>
+        <v/>
+      </c>
+      <c r="M120" s="1020">
+        <f>M117*M119</f>
+        <v/>
+      </c>
+      <c r="N120" s="1020">
+        <f>N117*N119</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="685" t="n"/>
+      <c r="B121" s="685" t="n"/>
+      <c r="C121" s="692" t="inlineStr">
+        <is>
+          <t>(-) Restructuring &amp; Other Cash Charges</t>
+        </is>
+      </c>
+      <c r="D121" s="693" t="n"/>
+      <c r="E121" s="693" t="n"/>
+      <c r="F121" s="693" t="n"/>
+      <c r="G121" s="954" t="n"/>
+      <c r="H121" s="955" t="n"/>
+      <c r="I121" s="954" t="n"/>
+      <c r="J121" s="1033" t="n">
+        <v>-125</v>
+      </c>
+      <c r="K121" s="1033" t="n">
+        <v>-100</v>
+      </c>
+      <c r="L121" s="1033" t="n">
+        <v>-50</v>
+      </c>
+      <c r="M121" s="1033" t="n">
+        <v>-40</v>
+      </c>
+      <c r="N121" s="1033" t="n">
+        <v>-40</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="685" t="n"/>
+      <c r="B122" s="685" t="n"/>
+      <c r="C122" s="706" t="inlineStr">
+        <is>
+          <t>EBIT (to FCF build)</t>
+        </is>
+      </c>
+      <c r="D122" s="707" t="n"/>
+      <c r="E122" s="707" t="n"/>
+      <c r="F122" s="707" t="n"/>
+      <c r="G122" s="707" t="n"/>
+      <c r="H122" s="961" t="n"/>
+      <c r="I122" s="962" t="n"/>
+      <c r="J122" s="1034">
+        <f>J120+J121</f>
+        <v/>
+      </c>
+      <c r="K122" s="1034">
+        <f>K120+K121</f>
+        <v/>
+      </c>
+      <c r="L122" s="1034">
+        <f>L120+L121</f>
+        <v/>
+      </c>
+      <c r="M122" s="1034">
+        <f>M120+M121</f>
+        <v/>
+      </c>
+      <c r="N122" s="1034">
+        <f>N120+N121</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="685" t="n"/>
+      <c r="B123" s="685" t="n"/>
+      <c r="C123" s="886" t="inlineStr">
+        <is>
+          <t>Depreciation (% of Revenue)</t>
+        </is>
+      </c>
+      <c r="D123" s="685" t="n"/>
+      <c r="E123" s="685" t="n"/>
+      <c r="F123" s="685" t="n"/>
+      <c r="G123" s="685" t="n"/>
+      <c r="H123" s="685" t="n"/>
+      <c r="I123" s="685" t="n"/>
+      <c r="J123" s="1032" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="K123" s="1035">
+        <f>J123</f>
+        <v/>
+      </c>
+      <c r="L123" s="1035">
+        <f>K123</f>
+        <v/>
+      </c>
+      <c r="M123" s="1035">
+        <f>L123</f>
+        <v/>
+      </c>
+      <c r="N123" s="1035">
+        <f>M123</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="685" t="n"/>
+      <c r="B124" s="685" t="n"/>
+      <c r="C124" s="692" t="inlineStr">
+        <is>
+          <t>Depreciation</t>
+        </is>
+      </c>
+      <c r="D124" s="693" t="n"/>
+      <c r="E124" s="693" t="n"/>
+      <c r="F124" s="693" t="n"/>
+      <c r="G124" s="954" t="n"/>
+      <c r="H124" s="955" t="n"/>
+      <c r="I124" s="954" t="n"/>
+      <c r="J124" s="1020">
+        <f>J117*J123</f>
+        <v/>
+      </c>
+      <c r="K124" s="1020">
+        <f>K117*K123</f>
+        <v/>
+      </c>
+      <c r="L124" s="1020">
+        <f>L117*L123</f>
+        <v/>
+      </c>
+      <c r="M124" s="1020">
+        <f>M117*M123</f>
+        <v/>
+      </c>
+      <c r="N124" s="1020">
+        <f>N117*N123</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="685" t="n"/>
+      <c r="B125" s="685" t="n"/>
+      <c r="C125" s="886" t="inlineStr">
+        <is>
+          <t>Capex incl. Equipment on Operating Leases (% of Revenue)</t>
+        </is>
+      </c>
+      <c r="D125" s="685" t="n"/>
+      <c r="E125" s="685" t="n"/>
+      <c r="F125" s="685" t="n"/>
+      <c r="G125" s="685" t="n"/>
+      <c r="H125" s="685" t="n"/>
+      <c r="I125" s="685" t="n"/>
+      <c r="J125" s="1032" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="K125" s="1035">
+        <f>J125</f>
+        <v/>
+      </c>
+      <c r="L125" s="1035">
+        <f>K125</f>
+        <v/>
+      </c>
+      <c r="M125" s="1035">
+        <f>L125</f>
+        <v/>
+      </c>
+      <c r="N125" s="1035">
+        <f>M125</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="685" t="n"/>
+      <c r="B126" s="685" t="n"/>
+      <c r="C126" s="692" t="inlineStr">
+        <is>
+          <t>Capex incl. Equipment on Operating Leases</t>
+        </is>
+      </c>
+      <c r="D126" s="693" t="n"/>
+      <c r="E126" s="693" t="n"/>
+      <c r="F126" s="693" t="n"/>
+      <c r="G126" s="954" t="n"/>
+      <c r="H126" s="955" t="n"/>
+      <c r="I126" s="954" t="n"/>
+      <c r="J126" s="1020">
+        <f>-J117*J125</f>
+        <v/>
+      </c>
+      <c r="K126" s="1020">
+        <f>-K117*K125</f>
+        <v/>
+      </c>
+      <c r="L126" s="1020">
+        <f>-L117*L125</f>
+        <v/>
+      </c>
+      <c r="M126" s="1020">
+        <f>-M117*M125</f>
+        <v/>
+      </c>
+      <c r="N126" s="1020">
+        <f>-N117*N125</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="685" t="n"/>
+      <c r="B127" s="685" t="n"/>
+      <c r="C127" s="886" t="inlineStr">
+        <is>
+          <t>Operating NWC (% of Revenue)</t>
+        </is>
+      </c>
+      <c r="D127" s="685" t="n"/>
+      <c r="E127" s="685" t="n"/>
+      <c r="F127" s="685" t="n"/>
+      <c r="G127" s="685" t="n"/>
+      <c r="H127" s="685" t="n"/>
+      <c r="I127" s="685" t="n"/>
+      <c r="J127" s="1032" t="n">
+        <v>-0.027</v>
+      </c>
+      <c r="K127" s="1035">
+        <f>J127</f>
+        <v/>
+      </c>
+      <c r="L127" s="1035">
+        <f>K127</f>
+        <v/>
+      </c>
+      <c r="M127" s="1035">
+        <f>L127</f>
+        <v/>
+      </c>
+      <c r="N127" s="1035">
+        <f>M127</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="685" t="n"/>
+      <c r="B128" s="685" t="n"/>
+      <c r="C128" s="692" t="inlineStr">
+        <is>
+          <t>(-) Change in Operating NWC</t>
+        </is>
+      </c>
+      <c r="D128" s="693" t="n"/>
+      <c r="E128" s="693" t="n"/>
+      <c r="F128" s="693" t="n"/>
+      <c r="G128" s="954" t="n"/>
+      <c r="H128" s="955" t="n"/>
+      <c r="I128" s="954" t="n"/>
+      <c r="J128" s="1036" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" s="1020">
+        <f>-K127*(K117-J117)</f>
+        <v/>
+      </c>
+      <c r="L128" s="1020">
+        <f>-L127*(L117-K117)</f>
+        <v/>
+      </c>
+      <c r="M128" s="1020">
+        <f>-M127*(M117-L117)</f>
+        <v/>
+      </c>
+      <c r="N128" s="1020">
+        <f>-N127*(N117-M117)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="685" t="n"/>
+      <c r="B129" s="685" t="n"/>
+      <c r="C129" s="692" t="inlineStr">
+        <is>
+          <t>Adj. EBITDA (excl. IEEPA)</t>
+        </is>
+      </c>
+      <c r="D129" s="693" t="n"/>
+      <c r="E129" s="693" t="n"/>
+      <c r="F129" s="693" t="n"/>
+      <c r="G129" s="954" t="n"/>
+      <c r="H129" s="955" t="n"/>
+      <c r="I129" s="954" t="n"/>
+      <c r="J129" s="1030">
+        <f>J120+J124</f>
+        <v/>
+      </c>
+      <c r="K129" s="1030">
+        <f>K120+K124</f>
+        <v/>
+      </c>
+      <c r="L129" s="1030">
+        <f>L120+L124</f>
+        <v/>
+      </c>
+      <c r="M129" s="1030">
+        <f>M120+M124</f>
+        <v/>
+      </c>
+      <c r="N129" s="1030">
+        <f>N120+N124</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="685" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B130" s="685" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C130" s="886" t="inlineStr">
+        <is>
+          <t>Memo: Unlevered FCF Margin</t>
+        </is>
+      </c>
+      <c r="D130" s="685" t="n"/>
+      <c r="E130" s="685" t="n"/>
+      <c r="F130" s="685" t="n"/>
+      <c r="G130" s="685" t="n"/>
+      <c r="H130" s="685" t="n"/>
+      <c r="I130" s="685" t="n"/>
+      <c r="J130" s="1035">
+        <f>J13/J117</f>
+        <v/>
+      </c>
+      <c r="K130" s="1035">
+        <f>K13/K117</f>
+        <v/>
+      </c>
+      <c r="L130" s="1035">
+        <f>L13/L117</f>
+        <v/>
+      </c>
+      <c r="M130" s="1035">
+        <f>M13/M117</f>
+        <v/>
+      </c>
+      <c r="N130" s="1035">
+        <f>N13/N117</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
         <is>
           <t>End</t>
         </is>
@@ -28508,21 +29131,23 @@
         <v/>
       </c>
       <c r="B1" s="445">
-        <f>'[1]Cover Page'!A1</f>
+        <f>'Cover Page'!A1</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="C2" s="447">
-        <f>"$"&amp;'[1]Cover Page'!E16&amp;" Stock Performance"</f>
-        <v/>
+      <c r="C2" s="447" t="inlineStr">
+        <is>
+          <t>$XRX Stock Performance</t>
+        </is>
       </c>
       <c r="D2" s="447" t="n"/>
       <c r="E2" s="447" t="n"/>
       <c r="F2" s="447" t="n"/>
-      <c r="G2" s="448">
-        <f>'[1]Cover Page'!C2</f>
-        <v/>
+      <c r="G2" s="448" t="inlineStr">
+        <is>
+          <t>Xerox Holdings Corporation</t>
+        </is>
       </c>
       <c r="H2" s="449" t="n"/>
       <c r="I2" s="449" t="n"/>
@@ -28585,7 +29210,7 @@
       </c>
       <c r="D6" s="456" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>XRX</t>
         </is>
       </c>
       <c r="E6" s="456" t="inlineStr">
@@ -28595,7 +29220,7 @@
       </c>
       <c r="F6" s="456" t="inlineStr">
         <is>
-          <t>FRSH Return</t>
+          <t>XRX Return</t>
         </is>
       </c>
       <c r="G6" s="456" t="inlineStr">

</xml_diff>